<commit_message>
feature ;- Create Mega Event excel update after run the flow add mega event
</commit_message>
<xml_diff>
--- a/resources/Create_MegaEvent_Prod.xlsx
+++ b/resources/Create_MegaEvent_Prod.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\ProjectM\MYBharat-Automation\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{44C7E934-D522-4E4D-A5A8-FFF584595F24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2F1AB7D-46BF-4150-9D59-970E642442BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9AF48352-515E-4DC0-AA5C-BFF759C0F978}"/>
+    <workbookView xWindow="6552" yWindow="5232" windowWidth="17280" windowHeight="8880" xr2:uid="{9AF48352-515E-4DC0-AA5C-BFF759C0F978}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Mega_Event_Name</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>Automation Mega Event 1528</t>
+  </si>
+  <si>
+    <t>Automation Mega Event 3888</t>
   </si>
 </sst>
 </file>
@@ -432,10 +435,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A22B34-7537-40DA-B43C-DE3D9D0AA4E0}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="16.21875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="24.21875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -443,39 +446,44 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s" s="0">
         <v>1</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s" s="0">
         <v>2</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s" s="0">
         <v>3</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s" s="0">
         <v>4</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s" s="0">
         <v>5</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s" s="0">
         <v>6</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s" s="0">
         <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feature:- modified the mega event name, changes in photo upload in past mega event
</commit_message>
<xml_diff>
--- a/resources/Create_MegaEvent_Prod.xlsx
+++ b/resources/Create_MegaEvent_Prod.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>Mega_Event_Name</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>Automation Mega Event 3888</t>
+  </si>
+  <si>
+    <t>Seva Se Seekhen</t>
   </si>
 </sst>
 </file>
@@ -435,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A22B34-7537-40DA-B43C-DE3D9D0AA4E0}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="24.21875"/>
@@ -486,6 +489,16 @@
         <v>8</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- changes in flow and fix time issue
</commit_message>
<xml_diff>
--- a/resources/Create_MegaEvent_Prod.xlsx
+++ b/resources/Create_MegaEvent_Prod.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="11">
   <si>
     <t>Mega_Event_Name</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>Seva Se Seekhen</t>
+  </si>
+  <si>
+    <t>Seeva See Seekhen</t>
   </si>
 </sst>
 </file>
@@ -438,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9A22B34-7537-40DA-B43C-DE3D9D0AA4E0}">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="24.21875"/>
@@ -499,6 +502,21 @@
         <v>9</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature :- changes in all module xml
</commit_message>
<xml_diff>
--- a/resources/Create_MegaEvent_Prod.xlsx
+++ b/resources/Create_MegaEvent_Prod.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="1">
   <si>
     <t>Seeva See Seekhen</t>
   </si>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="24.21875"/>
@@ -572,6 +572,26 @@
         <v>0</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>